<commit_message>
Tabulka inzeratov: styri nove prihlasky a stlpec dokladov
Doplnene Barux, Istropolitana Ogilvy, LICI Advertising a i-Step,
vsetky so zaznamom o tom, kedy a cez ktory kanal sa prihlasila.

Dva datumy boli len poznamka pre nu samu ("doplnit", "over si"),
teraz su to skutocne datumy: Kempelenov 1. 8., High5 a Expresta 4. 8.

Stlpec Doklad pre urad prace bol prazdny vo vsetkych riadkoch.
Ku kazdej odoslanej prihlaske je teraz napisane, co si k nej treba
odlozit, podla kanala: potvrdenie z Profesie, z Prace za rohom,
alebo vlastny odoslany e-mail pri Pretlaku, vzdy plus PDF inzeratu.
Pri Kempelenove a High5 staci e-mail s odmietnutim.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRJ8GE4B9NBudRKNSE36EN
</commit_message>
<xml_diff>
--- a/career/Viktoria-hladanie-prace.xlsx
+++ b/career/Viktoria-hladanie-prace.xlsx
@@ -116,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -162,6 +162,9 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3397,7 +3400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3504,13 +3507,15 @@
           <t>DTP a príprava do tlače, presne tvoja priemyslovka. Overené 18. 8., inzerát stále beží a v texte píšu, že nemusíš byť profík.</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="23" t="inlineStr">
         <is>
           <t>pracazarohom.sk/dl/jd/PROF-6a4718b0-822d-4a57-9545-17e78e63c442</t>
         </is>
       </c>
+      <c r="I5" s="23" t="n"/>
+      <c r="J5" s="23" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -3538,13 +3543,15 @@
           <t>Sadzba dlhých dokumentov v InDesigne. Overené 18. 8., beží na ich vlastnom kariérnom webe. 4 dni práca, 4 dni voľno, 32 hodín týždenne.</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="23" t="inlineStr">
         <is>
           <t>freshfields.wd3.myworkdayjobs.com, pozícia R-06803-1</t>
         </is>
       </c>
+      <c r="I6" s="23" t="n"/>
+      <c r="J6" s="23" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -3582,14 +3589,19 @@
           <t>11. 8. 2026</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="23" t="inlineStr">
         <is>
           <t>pracazarohom.sk</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="23" t="inlineStr">
         <is>
           <t>Cez Prácu za rohom</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + potvrdenie o prihlásení z Práce za rohom</t>
         </is>
       </c>
     </row>
@@ -3626,17 +3638,22 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>doplniť</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
+          <t>1. 8. 2026</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
         <is>
           <t>profesia.sk</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="23" t="inlineStr">
         <is>
           <t>Cez Profesiu</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + e-mail s odmietnutím</t>
         </is>
       </c>
     </row>
@@ -3666,8 +3683,11 @@
           <t>Kníhtlačiareň, obsahovo ideálne, geograficky ďaleko</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="23" t="n"/>
+      <c r="I9" s="23" t="n"/>
+      <c r="J9" s="23" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -3695,8 +3715,11 @@
           <t>To isté bližšie k Trnave, horšie platené</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="23" t="n"/>
+      <c r="I10" s="23" t="n"/>
+      <c r="J10" s="23" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -3724,8 +3747,11 @@
           <t>Tlačiareň, široké rozpätie</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="23" t="n"/>
+      <c r="I11" s="23" t="n"/>
+      <c r="J11" s="23" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -3760,17 +3786,22 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>utorok 4. 8. 2026 (over si)</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
+          <t>4. 8. 2026</t>
+        </is>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
         <is>
           <t>pretlak.com</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="23" t="inlineStr">
         <is>
           <t>Cez Pretlak</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + e-mail s odmietnutím</t>
         </is>
       </c>
     </row>
@@ -3810,14 +3841,19 @@
           <t>11. 8. 2026</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="23" t="inlineStr">
         <is>
           <t>profesia.sk</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="23" t="inlineStr">
         <is>
           <t>Cez Profesiu a mail na kariera@sng.sk</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + potvrdenie z Profesie + odoslaný mail na kariera@sng.sk</t>
         </is>
       </c>
     </row>
@@ -3854,17 +3890,22 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>utorok 4. 8. 2026 (over si)</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
+          <t>4. 8. 2026</t>
+        </is>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
         <is>
           <t>profesia.sk</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="23" t="inlineStr">
         <is>
           <t>Cez Profesiu</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + potvrdzujúci e-mail z Profesie</t>
         </is>
       </c>
     </row>
@@ -3904,14 +3945,19 @@
           <t>11. 8. 2026</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="23" t="inlineStr">
         <is>
           <t>pracazarohom.sk</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="23" t="inlineStr">
         <is>
           <t>Cez Prácu za rohom</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + potvrdenie o prihlásení z Práce za rohom</t>
         </is>
       </c>
     </row>
@@ -3951,251 +3997,513 @@
           <t>14. 8. 2026</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="23" t="inlineStr">
         <is>
           <t>pretlak.com</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="23" t="inlineStr">
         <is>
           <t>Cez Pretlak</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + odoslaný e-mail z Odoslanej pošty</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Motion &amp; Graphic Designer</t>
+          <t>Mid / senior grafický dizajnér</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>KLARSTEIN (Berlin Brands Group)</t>
+          <t>Barux s. r. o.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Bratislava, Grösslingová</t>
+          <t>Bratislava</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>od 1 600 €</t>
+          <t>1 900 €</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Motion, strih videa a AI nástroje. Nežiadajú počet rokov praxe.</t>
+          <t>Kreatívne grafické štúdio</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>nie</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>profesia.sk/praca/klarstein-berlin-brands-group/O5331654</t>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>14. 9. 2026</t>
+        </is>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>profesia.sk</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>Cez Profesiu</t>
+        </is>
+      </c>
+      <c r="J17" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + potvrdzujúci e-mail z Profesie</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Referent marketingu, obsah pre sociálne siete</t>
+          <t>Art Director</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>dm drogerie markt</t>
+          <t>Istropolitana Ogilvy</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Bratislava, Záhradnícka</t>
+          <t>Bratislava</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>2 196 €</t>
+          <t>od 2 000 €</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Presne to, čo robíš pre ShapelesAi. Najlepšie platené z celého zoznamu.</t>
+          <t>Kreatívna reklamná agentúra</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>nie</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>profesia.sk/praca/dm-drogerie-markt/O5335002</t>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>14. 9. 2026</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>pretlak.com</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>Cez Pretlak</t>
+        </is>
+      </c>
+      <c r="J18" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + odoslaný e-mail z Odoslanej pošty</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Marketingový špecialista junior</t>
+          <t>Grafický dizajnér mid/senior</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>MediaTech Central Europe</t>
+          <t>LIČI Advertising</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Bratislava, Drieňová 34</t>
+          <t>Bratislava, Ružinov</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>od 1 500 €</t>
+          <t>od 2 000 €</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Junior pozícia, marketing s grafikou.</t>
+          <t>Reklamná agentúra</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>nie</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="n"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>profesia.sk/praca/mediatech-central-europe/O5333256</t>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>17. 9. 2026</t>
+        </is>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>pretlak.com</t>
+        </is>
+      </c>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>Cez Pretlak</t>
+        </is>
+      </c>
+      <c r="J19" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + odoslaný e-mail z Odoslanej pošty</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Graphic Designer</t>
+          <t>Grafický dizajnér mid</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Premedix</t>
+          <t>i-Step</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Bratislava, Panenská 7</t>
+          <t>Bratislava, hybrid</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>1 800 €</t>
+          <t>od 1 600 €, faktúra</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Print aj digitál. Žiadajú 2 až 3 roky praxe, výber je na tri kolá so zadaním.</t>
+          <t>Full service marketingová agentúra. Brand identity, kampane, social aj print. Žiadajú Adobe aj Figmu, plus body za motion, AI nástroje a ilustráciu.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>nie</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>profesia.sk/praca/premedix/O5333707</t>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>17. 9. 2026</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>pretlak.com</t>
+        </is>
+      </c>
+      <c r="I20" s="23" t="inlineStr">
+        <is>
+          <t>Cez Pretlak</t>
+        </is>
+      </c>
+      <c r="J20" s="23" t="inlineStr">
+        <is>
+          <t>PDF inzerátu + odoslaný e-mail z Odoslanej pošty</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>Motion &amp; Graphic Designer</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>KLARSTEIN (Berlin Brands Group)</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, Grösslingová</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>od 1 600 €</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Motion, strih videa a AI nástroje. Nežiadajú počet rokov praxe.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>profesia.sk/praca/klarstein-berlin-brands-group/O5331654</t>
+        </is>
+      </c>
+      <c r="I21" s="23" t="n"/>
+      <c r="J21" s="23" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Referent marketingu, obsah pre sociálne siete</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>dm drogerie markt</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, Záhradnícka</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>2 196 €</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Presne to, čo robíš pre ShapelesAi. Najlepšie platené z celého zoznamu.</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="23" t="inlineStr">
+        <is>
+          <t>profesia.sk/praca/dm-drogerie-markt/O5335002</t>
+        </is>
+      </c>
+      <c r="I22" s="23" t="n"/>
+      <c r="J22" s="23" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Marketingový špecialista junior</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>MediaTech Central Europe</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, Drieňová 34</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>od 1 500 €</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Junior pozícia, marketing s grafikou.</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="23" t="inlineStr">
+        <is>
+          <t>profesia.sk/praca/mediatech-central-europe/O5333256</t>
+        </is>
+      </c>
+      <c r="I23" s="23" t="n"/>
+      <c r="J23" s="23" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Graphic Designer</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Premedix</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Bratislava, Panenská 7</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>1 800 €</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Print aj digitál. Žiadajú 2 až 3 roky praxe, výber je na tri kolá so zadaním.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="23" t="inlineStr">
+        <is>
+          <t>profesia.sk/praca/premedix/O5333707</t>
+        </is>
+      </c>
+      <c r="I24" s="23" t="n"/>
+      <c r="J24" s="23" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
           <t>Grafik / kreatívny pracovník</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>SLARA</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Bratislava, Gagarinova</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>1 500 – 2 100 €</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Agentúra. Žiadajú 3 roky praxe a je to na živnosť. Bez portfólia CV nečítajú.</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>nie</t>
         </is>
       </c>
-      <c r="G21" s="4" t="n"/>
-      <c r="H21" t="inlineStr">
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="23" t="inlineStr">
         <is>
           <t>profesia.sk/praca/slara/O3961268</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr"/>
-      <c r="B24" s="4" t="inlineStr"/>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr"/>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr"/>
-      <c r="B25" s="4" t="inlineStr"/>
-      <c r="C25" s="4" t="inlineStr"/>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="4" t="inlineStr"/>
+      <c r="I25" s="23" t="n"/>
+      <c r="J25" s="23" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr"/>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr"/>
-      <c r="F26" s="4" t="inlineStr"/>
-      <c r="G26" s="4" t="inlineStr"/>
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="23" t="n"/>
+      <c r="I26" s="23" t="n"/>
+      <c r="J26" s="23" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="23" t="n"/>
+      <c r="C27" s="23" t="n"/>
+      <c r="D27" s="23" t="n"/>
+      <c r="E27" s="23" t="n"/>
+      <c r="F27" s="23" t="n"/>
+      <c r="G27" s="23" t="n"/>
+      <c r="H27" s="23" t="n"/>
+      <c r="I27" s="23" t="n"/>
+      <c r="J27" s="23" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="23" t="n"/>
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
+      <c r="F28" s="23" t="n"/>
+      <c r="G28" s="23" t="n"/>
+      <c r="H28" s="23" t="n"/>
+      <c r="I28" s="23" t="n"/>
+      <c r="J28" s="23" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="23" t="n"/>
+      <c r="C29" s="23" t="n"/>
+      <c r="D29" s="23" t="n"/>
+      <c r="E29" s="23" t="n"/>
+      <c r="F29" s="23" t="n"/>
+      <c r="G29" s="23" t="n"/>
+      <c r="H29" s="23" t="n"/>
+      <c r="I29" s="23" t="n"/>
+      <c r="J29" s="23" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="23" t="n"/>
+      <c r="C30" s="23" t="n"/>
+      <c r="D30" s="23" t="n"/>
+      <c r="E30" s="23" t="n"/>
+      <c r="F30" s="23" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="23" t="n"/>
+      <c r="I30" s="23" t="n"/>
+      <c r="J30" s="23" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="23" t="n"/>
+      <c r="C31" s="23" t="n"/>
+      <c r="D31" s="23" t="n"/>
+      <c r="E31" s="23" t="n"/>
+      <c r="F31" s="23" t="n"/>
+      <c r="G31" s="23" t="n"/>
+      <c r="H31" s="23" t="n"/>
+      <c r="I31" s="23" t="n"/>
+      <c r="J31" s="23" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="n"/>
+      <c r="B32" s="23" t="n"/>
+      <c r="C32" s="23" t="n"/>
+      <c r="D32" s="23" t="n"/>
+      <c r="E32" s="23" t="n"/>
+      <c r="F32" s="23" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="23" t="n"/>
+      <c r="I32" s="23" t="n"/>
+      <c r="J32" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4208,7 +4516,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"áno,nie"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>